<commit_message>
feat(api): compact utility statement PDF with min kWh and tight footer spacing
Size PDF pages to sheet content via singlePageSheets and custom paper twips, show minimum kWh when billed usage exceeds actual, and collapse loose footer rows around Cara Pembayaran.
</commit_message>
<xml_diff>
--- a/apps/api/assets/utility-statement.xlsx
+++ b/apps/api/assets/utility-statement.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
     <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">Sheet1!$A2:$M51</definedName>
     <definedName name="Title">Sheet1!$G$3</definedName>
     <definedName name="GuestName">Sheet1!$D$5</definedName>
     <definedName name="GuestPhone">Sheet1!$D$6</definedName>
@@ -22,6 +22,7 @@
     <definedName name="ElecStartKwh">Sheet1!$F$14</definedName>
     <definedName name="ElecEndKwh">Sheet1!$I$14</definedName>
     <definedName name="ElecActualUsage">Sheet1!$F$15</definedName>
+    <definedName name="ElecMinKwh">Sheet1!$F$16</definedName>
     <definedName name="ElecBilledKwh">Sheet1!$F$17</definedName>
     <definedName name="ElecChargeKwh">Sheet1!$F$19</definedName>
     <definedName name="ElecRate">Sheet1!$I$19</definedName>
@@ -38,18 +39,16 @@
     <definedName name="PeriodSubtotal">Sheet1!$L$33</definedName>
     <definedName name="AdminAmount">Sheet1!$L$34</definedName>
     <definedName name="DueAmount">Sheet1!$L$35</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Sheet1'!$A2:$M51</definedName>
   </definedNames>
-  <calcPr/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{D0CA8CA8-9F24-4464-BF8E-62219DCF47F9}"/>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
-  <si>
-    <t xml:space="preserve">BILLING STATEMENT</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="53">
+  <si>
+    <t>BILLING STATEMENT</t>
   </si>
   <si>
     <t>Nama</t>
@@ -61,7 +60,7 @@
     <t>Telpon</t>
   </si>
   <si>
-    <t xml:space="preserve">No Unit</t>
+    <t>No Unit</t>
   </si>
   <si>
     <t>Periode</t>
@@ -82,13 +81,13 @@
     <t>Deskripsi</t>
   </si>
   <si>
-    <t xml:space="preserve">Biaya (Rp)</t>
+    <t>Biaya (Rp)</t>
   </si>
   <si>
     <t>Maintenance</t>
   </si>
   <si>
-    <t xml:space="preserve">Listrik (Electricity)</t>
+    <t>Listrik (Electricity)</t>
   </si>
   <si>
     <t>Konsumsi</t>
@@ -100,10 +99,10 @@
     <t>s.d</t>
   </si>
   <si>
-    <t xml:space="preserve">Pemakaian / Usage</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Minimum pakai</t>
+    <t>Pemakaian / Usage</t>
+  </si>
+  <si>
+    <t>Minimum pakai</t>
   </si>
   <si>
     <t>jam</t>
@@ -115,22 +114,22 @@
     <t>kVA</t>
   </si>
   <si>
-    <t xml:space="preserve">Tagihan terhutang</t>
+    <t>Tagihan terhutang</t>
   </si>
   <si>
     <t>Rp/kWh</t>
   </si>
   <si>
-    <t xml:space="preserve">Area Publik (PJU)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Handling Charge</t>
+    <t>Area Publik (PJU)</t>
+  </si>
+  <si>
+    <t>Handling Charge</t>
   </si>
   <si>
     <t>Rp</t>
   </si>
   <si>
-    <t xml:space="preserve">Air Bersih (Water Consumption)</t>
+    <t>Air Bersih (Water Consumption)</t>
   </si>
   <si>
     <r>
@@ -173,22 +172,22 @@
     <t>konstan</t>
   </si>
   <si>
-    <t xml:space="preserve">Pemeliharaan Meter</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hasil Akhir Tagihan :</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tagihan Bulan ini</t>
+    <t>Pemeliharaan Meter</t>
+  </si>
+  <si>
+    <t>Hasil Akhir Tagihan :</t>
+  </si>
+  <si>
+    <t>Tagihan Bulan ini</t>
   </si>
   <si>
     <t>Admin</t>
   </si>
   <si>
-    <t xml:space="preserve">Tagihan yang harus dibayar saat ini adalah</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Catatan :</t>
+    <t>Tagihan yang harus dibayar saat ini adalah</t>
+  </si>
+  <si>
+    <t>Catatan :</t>
   </si>
   <si>
     <r>
@@ -196,7 +195,7 @@
         <color theme="1"/>
         <rFont val="Calibri"/>
       </rPr>
-      <t xml:space="preserve">- Tanggal Jatuh tempo adalah tanggal 14 setiap bulannya. Pembayaran telat dikenakan denda 1</t>
+      <t>- Tanggal Jatuh tempo adalah tanggal 14 setiap bulannya. Pembayaran telat dikenakan denda 1</t>
     </r>
     <r>
       <rPr>
@@ -214,37 +213,37 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">Cara Pembayaran</t>
+    <t>Cara Pembayaran</t>
   </si>
   <si>
     <t xml:space="preserve">: </t>
   </si>
   <si>
-    <t xml:space="preserve">Pembayaran dapat ditransfer ke rekening berikut :</t>
+    <t>Pembayaran dapat ditransfer ke rekening berikut :</t>
   </si>
   <si>
     <t xml:space="preserve">Nama Bank </t>
   </si>
   <si>
-    <t xml:space="preserve">BANK RAKYAT INDONESIA  (BRI)</t>
+    <t>BANK RAKYAT INDONESIA  (BRI)</t>
   </si>
   <si>
     <t>A.N</t>
   </si>
   <si>
-    <t xml:space="preserve">PERUMNAS PROJECT SUKARAMAI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No. Rek</t>
+    <t>PERUMNAS PROJECT SUKARAMAI</t>
+  </si>
+  <si>
+    <t>No. Rek</t>
   </si>
   <si>
     <t>036701001560300</t>
   </si>
   <si>
-    <t xml:space="preserve">- Apabila penghuni belum melunasi tagihan, maka pengelola berhak melakukan pemutusan sementara</t>
-  </si>
-  <si>
-    <t xml:space="preserve">- Surat tagihan ini adalah cetakan komputer dan tidak memerlukan tanda tangan</t>
+    <t>- Apabila penghuni belum melunasi tagihan, maka pengelola berhak melakukan pemutusan sementara</t>
+  </si>
+  <si>
+    <t>- Surat tagihan ini adalah cetakan komputer dan tidak memerlukan tanda tangan</t>
   </si>
   <si>
     <t xml:space="preserve">- Pembayaran hanya di terima apabila melalui no rekening di atas. </t>
@@ -276,13 +275,13 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">- Jika tidak mengirim bukti pembayaran, maka dianggap belum melakukan pembayaran</t>
+    <t>- Jika tidak mengirim bukti pembayaran, maka dianggap belum melakukan pembayaran</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="6">
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* (#,##0.00);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="D/M/YYYY"/>
@@ -291,12 +290,13 @@
     <numFmt numFmtId="168" formatCode="dd/mm/yy"/>
     <numFmt numFmtId="169" formatCode="0.0"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
-      <sz val="11.000000"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <color theme="1"/>
@@ -305,8 +305,8 @@
     <font>
       <b/>
       <u/>
-      <sz val="18.000000"/>
       <color theme="1"/>
+      <sz val="18"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -315,26 +315,26 @@
     </font>
     <font>
       <b/>
-      <sz val="11.000000"/>
       <color theme="1"/>
+      <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
       <u/>
-      <sz val="11.000000"/>
       <color theme="1"/>
+      <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <sz val="11.000000"/>
       <color theme="1"/>
+      <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="15.000000"/>
       <color theme="1"/>
+      <sz val="15"/>
       <name val="Calibri"/>
     </font>
     <font/>
@@ -350,20 +350,20 @@
     </font>
     <font>
       <b/>
-      <sz val="12.000000"/>
       <color theme="1"/>
+      <sz val="12"/>
       <name val="Calibri"/>
     </font>
     <font>
       <u/>
-      <sz val="9.000000"/>
       <color theme="1"/>
+      <sz val="9"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-      <sz val="11.000000"/>
       <color indexed="2"/>
+      <sz val="11"/>
       <name val="Calibri"/>
     </font>
   </fonts>
@@ -381,13 +381,13 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="20">
     <border>
-      <left style="none"/>
-      <right style="none"/>
-      <top style="none"/>
-      <bottom style="none"/>
-      <diagonal style="none"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
     </border>
     <border>
       <left style="medium">
@@ -434,6 +434,13 @@
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <left style="none"/>
+      <right style="none"/>
+      <top style="none"/>
+      <bottom style="none"/>
+      <diagonal style="none"/>
     </border>
     <border>
       <left/>
@@ -585,136 +592,136 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="71">
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="2" fillId="0" borderId="4" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="2" fillId="0" borderId="5" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="6" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf fontId="1" fillId="0" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="4" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="5" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf fontId="6" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="6" fillId="0" borderId="8" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf fontId="6" fillId="0" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="165" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf fontId="4" fillId="0" borderId="7" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="7" fillId="0" borderId="9" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="7" fillId="0" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="7" fillId="0" borderId="10" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="7" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="4" fillId="0" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="6" fillId="0" borderId="8" numFmtId="166" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf fontId="6" fillId="0" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="8" fillId="0" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="11" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="5" fillId="0" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="6" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf fontId="6" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="6" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf fontId="4" fillId="0" borderId="8" numFmtId="165" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="8" numFmtId="167" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf fontId="4" fillId="0" borderId="8" numFmtId="167" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="6" fillId="0" borderId="0" numFmtId="168" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="9" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf fontId="9" fillId="0" borderId="0" numFmtId="167" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="9" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf fontId="9" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="1" fillId="0" borderId="0" numFmtId="169" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf fontId="10" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="169" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="169" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="167" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf fontId="6" fillId="0" borderId="0" numFmtId="167" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf fontId="10" fillId="0" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="3" fillId="0" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="3" fillId="0" borderId="8" numFmtId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf fontId="6" fillId="0" borderId="8" numFmtId="167" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="12" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="9" fillId="0" borderId="12" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="4" fillId="0" borderId="12" numFmtId="167" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="9" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="9" fillId="0" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="4" fillId="0" borderId="0" numFmtId="167" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="4" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="5" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="6" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="3" fillId="0" borderId="8" numFmtId="164" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf fontId="11" fillId="0" borderId="8" numFmtId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="11" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="12" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf fontId="4" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="3" fillId="0" borderId="8" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="1" fillId="0" borderId="13" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="13" fillId="0" borderId="8" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="14" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="9" fillId="2" borderId="15" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="15" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="16" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="17" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="1" fillId="0" borderId="18" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1211,29 +1218,31 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
-    <outlinePr applyStyles="0" summaryBelow="0" summaryRight="0" showOutlineSymbols="1"/>
-    <pageSetUpPr autoPageBreaks="1" fitToPage="1"/>
+    <pageSetUpPr fitToPage="1"/>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr defaultColWidth="12.630000000000001" defaultRowHeight="15.75" customHeight="1"/>
+  <dimension ref="A1:M52"/>
+  <sheetFormatPr defaultRowHeight="15.75" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="12.63" customHeight="1"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="3.6299999999999999"/>
-    <col customWidth="1" min="2" max="2" width="7.6299999999999999"/>
-    <col customWidth="1" min="3" max="3" width="1.6299999999999999"/>
-    <col customWidth="1" min="4" max="4" width="16.25"/>
-    <col customWidth="1" min="5" max="5" width="1.8799999999999999"/>
-    <col customWidth="1" min="6" max="6" width="8.8800000000000008"/>
-    <col customWidth="1" min="7" max="7" width="5.25"/>
-    <col customWidth="1" min="8" max="8" width="6.25"/>
-    <col customWidth="1" min="9" max="9" width="6.6299999999999999"/>
-    <col customWidth="1" min="10" max="10" width="7.1299999999999999"/>
-    <col customWidth="1" min="11" max="11" width="3"/>
-    <col customWidth="1" min="12" max="12" width="12.880000000000001"/>
-    <col customWidth="1" min="13" max="13" width="10.00390625"/>
+    <col min="1" max="1" width="3.63" customWidth="1"/>
+    <col min="2" max="2" width="7.63" customWidth="1"/>
+    <col min="3" max="3" width="1.63" customWidth="1"/>
+    <col min="4" max="4" width="16.25" customWidth="1"/>
+    <col min="5" max="5" width="1.88" customWidth="1"/>
+    <col min="6" max="6" width="8.88" customWidth="1"/>
+    <col min="7" max="7" width="5.25" customWidth="1"/>
+    <col min="8" max="8" width="6.25" customWidth="1"/>
+    <col min="9" max="9" width="6.63" customWidth="1"/>
+    <col min="10" max="10" width="7.13" customWidth="1"/>
+    <col min="11" max="11" width="3" customWidth="1"/>
+    <col min="12" max="12" width="12.88" customWidth="1"/>
+    <col min="13" max="13" width="10.00390625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" ht="23.25" customHeight="1">
+    <row r="1" spans="4:4" x14ac:dyDescent="0.25"/>
+    <row r="2" ht="23.25" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1248,7 +1257,7 @@
       <c r="L2" s="2"/>
       <c r="M2" s="3"/>
     </row>
-    <row r="3" ht="23.25" customHeight="1">
+    <row r="3" ht="23.25" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>0</v>
       </c>
@@ -1265,7 +1274,7 @@
       <c r="L3" s="5"/>
       <c r="M3" s="6"/>
     </row>
-    <row r="4">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="7"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -1280,7 +1289,7 @@
       <c r="L4" s="8"/>
       <c r="M4" s="10"/>
     </row>
-    <row r="5">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="7"/>
       <c r="B5" s="11" t="s">
         <v>1</v>
@@ -1299,7 +1308,7 @@
       <c r="L5" s="8"/>
       <c r="M5" s="10"/>
     </row>
-    <row r="6" ht="20.25" customHeight="1">
+    <row r="6" ht="20.25" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="7"/>
       <c r="B6" s="13" t="s">
         <v>3</v>
@@ -1318,7 +1327,7 @@
       <c r="L6" s="8"/>
       <c r="M6" s="10"/>
     </row>
-    <row r="7" ht="20.25" customHeight="1">
+    <row r="7" ht="20.25" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="7"/>
       <c r="B7" s="11" t="s">
         <v>4</v>
@@ -1339,7 +1348,7 @@
       <c r="L7" s="8"/>
       <c r="M7" s="10"/>
     </row>
-    <row r="8">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="7"/>
       <c r="B8" s="22" t="s">
         <v>5</v>
@@ -1360,7 +1369,7 @@
       <c r="L8" s="15"/>
       <c r="M8" s="10"/>
     </row>
-    <row r="9">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="26"/>
       <c r="B9" s="15" t="s">
         <v>7</v>
@@ -1383,7 +1392,7 @@
       <c r="L9" s="30"/>
       <c r="M9" s="10"/>
     </row>
-    <row r="10">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A10" s="7"/>
       <c r="B10" s="16"/>
       <c r="C10" s="8"/>
@@ -1398,7 +1407,7 @@
       <c r="L10" s="8"/>
       <c r="M10" s="10"/>
     </row>
-    <row r="11">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="7"/>
       <c r="B11" s="31" t="s">
         <v>9</v>
@@ -1419,7 +1428,7 @@
       </c>
       <c r="M11" s="10"/>
     </row>
-    <row r="12">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="7"/>
       <c r="B12" s="34">
         <f>F8</f>
@@ -1443,7 +1452,7 @@
       </c>
       <c r="M12" s="10"/>
     </row>
-    <row r="13">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="7"/>
       <c r="B13" s="16"/>
       <c r="C13" s="8"/>
@@ -1460,7 +1469,7 @@
       <c r="L13" s="8"/>
       <c r="M13" s="10"/>
     </row>
-    <row r="14">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="7"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -1489,7 +1498,7 @@
       <c r="L14" s="8"/>
       <c r="M14" s="10"/>
     </row>
-    <row r="15">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="7"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -1512,7 +1521,7 @@
       <c r="L15" s="8"/>
       <c r="M15" s="10"/>
     </row>
-    <row r="16" hidden="1">
+    <row r="16" hidden="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="7"/>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -1541,7 +1550,7 @@
       <c r="L16" s="8"/>
       <c r="M16" s="10"/>
     </row>
-    <row r="17" hidden="1">
+    <row r="17" hidden="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="7"/>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
@@ -1562,7 +1571,7 @@
       <c r="L17" s="36"/>
       <c r="M17" s="10"/>
     </row>
-    <row r="18">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="7"/>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
@@ -1577,7 +1586,7 @@
       <c r="L18" s="36"/>
       <c r="M18" s="10"/>
     </row>
-    <row r="19">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="7"/>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
@@ -1610,7 +1619,7 @@
       </c>
       <c r="M19" s="10"/>
     </row>
-    <row r="20">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="7"/>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
@@ -1633,7 +1642,7 @@
       </c>
       <c r="M20" s="10"/>
     </row>
-    <row r="21">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="7"/>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -1658,7 +1667,7 @@
       </c>
       <c r="M21" s="10"/>
     </row>
-    <row r="22">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="7"/>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -1677,7 +1686,7 @@
       </c>
       <c r="M22" s="10"/>
     </row>
-    <row r="23">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A23" s="7"/>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -1692,7 +1701,7 @@
       <c r="L23" s="36"/>
       <c r="M23" s="10"/>
     </row>
-    <row r="24">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="7"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -1709,7 +1718,7 @@
       <c r="L24" s="36"/>
       <c r="M24" s="10"/>
     </row>
-    <row r="25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="7"/>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -1738,7 +1747,7 @@
       <c r="L25" s="36"/>
       <c r="M25" s="10"/>
     </row>
-    <row r="26">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="7"/>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -1771,7 +1780,7 @@
       </c>
       <c r="M26" s="10"/>
     </row>
-    <row r="27">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="7"/>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -1796,7 +1805,7 @@
       </c>
       <c r="M27" s="10"/>
     </row>
-    <row r="28">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="7"/>
       <c r="B28" s="8"/>
       <c r="C28" s="8"/>
@@ -1821,7 +1830,7 @@
       </c>
       <c r="M28" s="10"/>
     </row>
-    <row r="29">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="7"/>
       <c r="B29" s="8"/>
       <c r="C29" s="8"/>
@@ -1846,7 +1855,7 @@
       </c>
       <c r="M29" s="10"/>
     </row>
-    <row r="30">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="7"/>
       <c r="B30" s="8"/>
       <c r="C30" s="8"/>
@@ -1865,7 +1874,7 @@
       </c>
       <c r="M30" s="10"/>
     </row>
-    <row r="31">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A31" s="7"/>
       <c r="B31" s="15"/>
       <c r="C31" s="15"/>
@@ -1880,7 +1889,7 @@
       <c r="L31" s="14"/>
       <c r="M31" s="10"/>
     </row>
-    <row r="32">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A32" s="7"/>
       <c r="B32" s="8"/>
       <c r="C32" s="8"/>
@@ -1897,7 +1906,7 @@
       <c r="L32" s="9"/>
       <c r="M32" s="10"/>
     </row>
-    <row r="33">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A33" s="7"/>
       <c r="B33" s="8"/>
       <c r="C33" s="8"/>
@@ -1918,7 +1927,7 @@
       </c>
       <c r="M33" s="10"/>
     </row>
-    <row r="34">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A34" s="7"/>
       <c r="B34" s="8"/>
       <c r="C34" s="8"/>
@@ -1939,7 +1948,7 @@
       </c>
       <c r="M34" s="10"/>
     </row>
-    <row r="35" ht="16.5" customHeight="1">
+    <row r="35" ht="16.5" customHeight="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A35" s="7"/>
       <c r="B35" s="8"/>
       <c r="C35" s="8"/>
@@ -1962,7 +1971,7 @@
       </c>
       <c r="M35" s="10"/>
     </row>
-    <row r="36">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A36" s="7"/>
       <c r="B36" s="8"/>
       <c r="C36" s="8"/>
@@ -1977,7 +1986,7 @@
       <c r="L36" s="8"/>
       <c r="M36" s="10"/>
     </row>
-    <row r="37">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
       <c r="B37" s="60" t="s">
         <v>37</v>
@@ -1994,7 +2003,7 @@
       <c r="L37" s="8"/>
       <c r="M37" s="10"/>
     </row>
-    <row r="38">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A38" s="7"/>
       <c r="B38" s="51" t="s">
         <v>38</v>
@@ -2011,7 +2020,7 @@
       <c r="L38" s="8"/>
       <c r="M38" s="10"/>
     </row>
-    <row r="39">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A39" s="7"/>
       <c r="B39" s="8"/>
       <c r="C39" s="8"/>
@@ -2026,7 +2035,7 @@
       <c r="L39" s="8"/>
       <c r="M39" s="10"/>
     </row>
-    <row r="40">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A40" s="7"/>
       <c r="B40" s="8"/>
       <c r="C40" s="8"/>
@@ -2045,7 +2054,7 @@
       <c r="L40" s="8"/>
       <c r="M40" s="10"/>
     </row>
-    <row r="41">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A41" s="7"/>
       <c r="B41" s="8"/>
       <c r="C41" s="10"/>
@@ -2062,7 +2071,7 @@
       <c r="L41" s="8"/>
       <c r="M41" s="10"/>
     </row>
-    <row r="42">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A42" s="7"/>
       <c r="B42" s="8"/>
       <c r="C42" s="10"/>
@@ -2083,7 +2092,7 @@
       <c r="L42" s="8"/>
       <c r="M42" s="10"/>
     </row>
-    <row r="43">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A43" s="7"/>
       <c r="B43" s="8"/>
       <c r="C43" s="10"/>
@@ -2104,7 +2113,7 @@
       <c r="L43" s="8"/>
       <c r="M43" s="10"/>
     </row>
-    <row r="44">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A44" s="7"/>
       <c r="B44" s="8"/>
       <c r="C44" s="10"/>
@@ -2125,7 +2134,7 @@
       <c r="L44" s="8"/>
       <c r="M44" s="10"/>
     </row>
-    <row r="45">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A45" s="7"/>
       <c r="B45" s="8"/>
       <c r="C45" s="8"/>
@@ -2140,7 +2149,7 @@
       <c r="L45" s="8"/>
       <c r="M45" s="10"/>
     </row>
-    <row r="46">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A46" s="7"/>
       <c r="B46" s="8"/>
       <c r="C46" s="8"/>
@@ -2155,7 +2164,7 @@
       <c r="L46" s="8"/>
       <c r="M46" s="10"/>
     </row>
-    <row r="47">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A47" s="7"/>
       <c r="B47" s="37" t="s">
         <v>48</v>
@@ -2172,7 +2181,7 @@
       <c r="L47" s="8"/>
       <c r="M47" s="10"/>
     </row>
-    <row r="48">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A48" s="7"/>
       <c r="B48" s="37" t="s">
         <v>49</v>
@@ -2189,7 +2198,7 @@
       <c r="L48" s="8"/>
       <c r="M48" s="10"/>
     </row>
-    <row r="49">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A49" s="7"/>
       <c r="B49" s="37" t="s">
         <v>50</v>
@@ -2206,7 +2215,7 @@
       <c r="L49" s="8"/>
       <c r="M49" s="10"/>
     </row>
-    <row r="50">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
       <c r="B50" s="37" t="s">
         <v>51</v>
@@ -2223,7 +2232,7 @@
       <c r="L50" s="8"/>
       <c r="M50" s="10"/>
     </row>
-    <row r="51">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A51" s="65"/>
       <c r="B51" s="66" t="s">
         <v>52</v>
@@ -2240,7 +2249,7 @@
       <c r="L51" s="67"/>
       <c r="M51" s="68"/>
     </row>
-    <row r="52">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A52" s="69"/>
       <c r="B52" s="70"/>
       <c r="C52" s="15"/>
@@ -2262,9 +2271,7 @@
     <mergeCell ref="D35:I35"/>
     <mergeCell ref="F44:I44"/>
   </mergeCells>
-  <printOptions headings="0" gridLines="0"/>
-  <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
-  <pageSetup paperSize="9" scale="100" firstPageNumber="1" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="1" errors="displayed" horizontalDpi="600" verticalDpi="600" copies="1"/>
-  <headerFooter/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="600" verticalDpi="600" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" usePrinterDefaults="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>